<commit_message>
Add NZ remittance letterhead and fix .eml not opening as a draft
- lib/companyInfo.ts: two letterhead profiles (AU/NZ), selected per
  supplier via the lookup file's IDCSCD country code. NZ differs from
  AU in entity name, no ABN, phone/fax labels, and total-row wording
  ("Total :" vs "Total this Debit :") — verified against a real NZ
  sample PDF, text-for-text match.
- lib/eml.ts: add X-Unsent: 1 header — without it Outlook opens a
  downloaded .eml as a read-only "received message" (no Send button,
  fields locked) instead of an editable draft.
- fixtures: add supplier 90006 (NZ) as the regression test case.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fixtures/sample-supplier-lookup.xlsx
+++ b/fixtures/sample-supplier-lookup.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -605,6 +605,44 @@
         </is>
       </c>
       <c r="I5" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>90006</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>KIWI SERVICES LTD</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>20</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>NZ</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>09 000 0006</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>accounts@kiwiservices.example.co.nz</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
         <is>
           <t>Valid</t>
         </is>

</xml_diff>

<commit_message>
Fix NZ bank export total line not being recognized
NZ writes "Total : <amount>" (no "this Debit"), unlike AU's "Total
this Debit : <amount>". The old regex only matched the AU wording, so
an NZ block never closed — the parser stayed stuck reading invoice
rows straight through the next block's header/GST/address noise,
misreading all of it as failed rows. Caught on a real 43-supplier NZ
file: 422 warnings, every supplier's statedTotal null.

Made "this Debit" optional in TOTAL_LINE. Regression test: supplier
90006 (NZ-formatted block, header wording reconstructed from the real
warning output) immediately followed by 90007 (AU) — proves both the
NZ close and no cascade into the next block. Verified against the live
app: 0 warnings, 0 mismatches across all 7 fixture suppliers.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fixtures/sample-supplier-lookup.xlsx
+++ b/fixtures/sample-supplier-lookup.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -643,6 +643,44 @@
         </is>
       </c>
       <c r="I6" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>90007</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>AFTER NZ CO</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>20</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>AU</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>03 9000 0007</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>ap@afternz.example.com</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
         <is>
           <t>Valid</t>
         </is>

</xml_diff>